<commit_message>
feat: refactor biblioteca documental y sincroniza dashboard
</commit_message>
<xml_diff>
--- a/pipeline/inputs/Listado_Maestro_2026__3_.xlsx
+++ b/pipeline/inputs/Listado_Maestro_2026__3_.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janto\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janto\OneDrive\Documentos\chicoorg\ERP CHICO\pipeline\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB322B0-D41A-4F00-97B0-3D8EF1D2FD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC63609-B5F7-4DDE-B368-90846B2F3ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{B7F87A59-495E-45F2-A6B5-6E41D0E42535}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15885" activeTab="4" xr2:uid="{B7F87A59-495E-45F2-A6B5-6E41D0E42535}"/>
   </bookViews>
   <sheets>
     <sheet name="1 Manuales - MGD - Est" sheetId="7" r:id="rId1"/>
@@ -513,7 +513,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="569">
   <si>
     <t>Estratégico</t>
   </si>
@@ -2219,6 +2219,9 @@
   </si>
   <si>
     <t>IL documentar el ANS para la firma asesores en lo referente a la parte contable</t>
+  </si>
+  <si>
+    <t>PRO-PROY-023312</t>
   </si>
 </sst>
 </file>
@@ -3707,7 +3710,7 @@
       </c>
       <c r="J3" s="52">
         <f ca="1">IF(I3="","",I3-TODAY())</f>
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K3" s="52" t="str">
         <f ca="1">IF(I3="","",IF(I3&lt;TODAY(),"Vencido",IF(I3-TODAY()&lt;=30,"Próximo a vencer","Vigente")))</f>
@@ -4135,7 +4138,7 @@
       </c>
       <c r="J10" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K10" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -4426,7 +4429,7 @@
       </c>
       <c r="J15" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K15" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -4596,7 +4599,7 @@
       </c>
       <c r="J18" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="K18" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -4779,7 +4782,7 @@
       </c>
       <c r="J21" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="K21" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -4861,7 +4864,7 @@
       </c>
       <c r="J22" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="K22" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -5093,7 +5096,7 @@
       </c>
       <c r="J26" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K26" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -5231,7 +5234,7 @@
       </c>
       <c r="J28" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K28" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -5415,7 +5418,7 @@
       </c>
       <c r="J31" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="K31" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -5499,7 +5502,7 @@
       </c>
       <c r="J32" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="K32" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -5960,7 +5963,7 @@
       </c>
       <c r="J40" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="K40" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -6310,7 +6313,7 @@
       </c>
       <c r="J46" s="52">
         <f t="shared" ca="1" si="0"/>
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="K46" s="52" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -11081,7 +11084,7 @@
     </row>
     <row r="86" spans="1:12">
       <c r="A86" s="77" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>551</v>

</xml_diff>